<commit_message>
adding script to sweep frequency and phase while tuning
</commit_message>
<xml_diff>
--- a/Hardware/Low Noise Pre-Amp/Low Noise Pre-Amp_BOM_v1.0.xlsx
+++ b/Hardware/Low Noise Pre-Amp/Low Noise Pre-Amp_BOM_v1.0.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jkell\Repositories\openEPR\Hardware\Low Noise Pre-Amp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5FF9CD61-3127-4709-B44D-68224E2C3A38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{083D05E3-30C5-461D-8C43-36C9C3A87DAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6174E856-FAF2-42DD-97B8-21F0085AEDC0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6174E856-FAF2-42DD-97B8-21F0085AEDC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Low Noise Pre-Amp_BOM_v1.0" sheetId="1" r:id="rId1"/>
@@ -417,7 +417,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -600,6 +600,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -773,11 +779,24 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1156,10 +1175,14 @@
   <dimension ref="A1:J15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="49.85546875" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" customWidth="1"/>
-    <col min="4" max="4" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" style="7" customWidth="1"/>
+    <col min="4" max="4" width="22.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="34.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="0" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="22.42578125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1169,10 +1192,10 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
@@ -1201,10 +1224,10 @@
       <c r="B2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="6">
         <v>12</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="3" t="s">
@@ -1230,10 +1253,10 @@
       <c r="B3" t="s">
         <v>17</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="7">
         <v>10</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F3" t="s">
@@ -1259,10 +1282,10 @@
       <c r="B4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="6">
         <v>3</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="6" t="s">
         <v>23</v>
       </c>
       <c r="F4" s="3" t="s">
@@ -1288,10 +1311,10 @@
       <c r="B5" t="s">
         <v>28</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="7">
         <v>1</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="7" t="s">
         <v>29</v>
       </c>
       <c r="F5" t="s">
@@ -1317,10 +1340,10 @@
       <c r="B6" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="6">
         <v>6</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="6" t="s">
         <v>35</v>
       </c>
       <c r="F6" s="3" t="s">
@@ -1346,10 +1369,10 @@
       <c r="B7" t="s">
         <v>41</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="7">
         <v>1</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="7">
         <v>220</v>
       </c>
       <c r="F7" t="s">
@@ -1375,10 +1398,10 @@
       <c r="B8" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="6">
         <v>2</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="6" t="s">
         <v>45</v>
       </c>
       <c r="F8" s="3" t="s">
@@ -1404,10 +1427,10 @@
       <c r="B9" t="s">
         <v>48</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="7">
         <v>5</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="7" t="s">
         <v>49</v>
       </c>
       <c r="F9" t="s">
@@ -1433,10 +1456,10 @@
       <c r="B10" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="6">
         <v>3</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="6" t="s">
         <v>53</v>
       </c>
       <c r="F10" s="3" t="s">
@@ -1455,26 +1478,26 @@
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11">
+    <row r="11" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="8">
         <v>2</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="4" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1485,10 +1508,10 @@
       <c r="B12" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="6">
         <v>2</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="6" t="s">
         <v>61</v>
       </c>
       <c r="F12" s="3" t="s">
@@ -1514,10 +1537,10 @@
       <c r="B13" t="s">
         <v>67</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="7">
         <v>1</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="7" t="s">
         <v>68</v>
       </c>
       <c r="F13" t="s">
@@ -1543,10 +1566,10 @@
       <c r="B14" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="6">
         <v>1</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="6" t="s">
         <v>74</v>
       </c>
       <c r="F14" s="3" t="s">
@@ -1572,10 +1595,10 @@
       <c r="B15" t="s">
         <v>80</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="7">
         <v>1</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="7" t="s">
         <v>81</v>
       </c>
       <c r="F15" t="s">

</xml_diff>